<commit_message>
Rearrange tracker to match live team roster and decouple team target
Roster now matches travnooker.com: Iyan, Harinder, Rihab Travnook,
Ibrahim Travnook, Chaimaa Benchohra, Saha Travnook, Alshimaa Ahmed,
Khozema Nogamawala (Bindhya Travnook is Team Leader, not a quota-carrying
agent). Added --team-target so the overall team goal (AED 170,000) can be
set independently of the sum of individual agent base targets (8 x 25,000
= 200,000) instead of always being their product.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DiEcNy7XAwqHLRjhRBareN
</commit_message>
<xml_diff>
--- a/trackers/SEPTEMBER_2026_TEAM_TRACKER_BINDHYA.xlsx
+++ b/trackers/SEPTEMBER_2026_TEAM_TRACKER_BINDHYA.xlsx
@@ -123,6 +123,9 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -139,9 +142,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -533,7 +533,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Team Lead: Bindhya   |   Monthly Target: AED 25,000 per agent   |   Working Days: 26   |   Mid-Month Checkpoint (by 12 Sep): AED 10,577 per agent</t>
+          <t>Team Lead: Bindhya Travnook   |   Team Target: AED 170,000   |   Per-Agent Base Target: AED 25,000   |   Working Days: 26   |   Mid-Month Checkpoint (by 12 Sep): AED 71,923 team</t>
         </is>
       </c>
     </row>
@@ -587,35 +587,34 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5">
-        <f>'Weekly Tracker'!C12</f>
-        <v/>
-      </c>
-      <c r="B6" s="5">
-        <f>'Weekly Tracker'!AS12</f>
-        <v/>
-      </c>
-      <c r="C6" s="5">
+      <c r="A6" s="5" t="n">
+        <v>170000</v>
+      </c>
+      <c r="B6" s="6">
+        <f>'Weekly Tracker'!AS14</f>
+        <v/>
+      </c>
+      <c r="C6" s="6">
         <f>A6-B6</f>
         <v/>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="6">
         <f>IFERROR(B6/A6,0)</f>
         <v/>
       </c>
-      <c r="E6" s="5">
-        <f>'Weekly Tracker'!D12+'Weekly Tracker'!L12</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>'Weekly Tracker'!J12+'Weekly Tracker'!S12</f>
-        <v/>
-      </c>
-      <c r="G6" s="5">
+      <c r="E6" s="6">
+        <f>ROUND(A6*11/26,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>'Weekly Tracker'!J14+'Weekly Tracker'!S14</f>
+        <v/>
+      </c>
+      <c r="G6" s="6">
         <f>ROUND(A6/26,0)</f>
         <v/>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="6">
         <f>IF(D6&gt;=1,"🟢 On Target",IF(D6&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
@@ -665,187 +664,187 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>SAHA</t>
-        </is>
-      </c>
-      <c r="B10" s="5">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Iyan</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
         <f>'Weekly Tracker'!C6</f>
         <v/>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="6">
         <f>'Weekly Tracker'!AS6</f>
         <v/>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="6">
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="6">
         <f>IFERROR(C10/B10,0)</f>
         <v/>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="6">
         <f>ROUND(B10/26,0)</f>
         <v/>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="6">
         <f>IF(E10&gt;=1,"🟢 On Target",IF(E10&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>IYAD</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Harinder</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
         <f>'Weekly Tracker'!C7</f>
         <v/>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="6">
         <f>'Weekly Tracker'!AS7</f>
         <v/>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="6">
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="6">
         <f>IFERROR(C11/B11,0)</f>
         <v/>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="6">
         <f>ROUND(B11/26,0)</f>
         <v/>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="6">
         <f>IF(E11&gt;=1,"🟢 On Target",IF(E11&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>RIHAB</t>
-        </is>
-      </c>
-      <c r="B12" s="5">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Rihab Travnook</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
         <f>'Weekly Tracker'!C8</f>
         <v/>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="6">
         <f>'Weekly Tracker'!AS8</f>
         <v/>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="6">
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="6">
         <f>IFERROR(C12/B12,0)</f>
         <v/>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="6">
         <f>ROUND(B12/26,0)</f>
         <v/>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="6">
         <f>IF(E12&gt;=1,"🟢 On Target",IF(E12&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>SHILPA</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Ibrahim Travnook</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
         <f>'Weekly Tracker'!C9</f>
         <v/>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="6">
         <f>'Weekly Tracker'!AS9</f>
         <v/>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="6">
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="6">
         <f>IFERROR(C13/B13,0)</f>
         <v/>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="6">
         <f>ROUND(B13/26,0)</f>
         <v/>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="6">
         <f>IF(E13&gt;=1,"🟢 On Target",IF(E13&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>ALSHIMAA</t>
-        </is>
-      </c>
-      <c r="B14" s="5">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Chaimaa Benchohra</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
         <f>'Weekly Tracker'!C10</f>
         <v/>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="6">
         <f>'Weekly Tracker'!AS10</f>
         <v/>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="6">
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="6">
         <f>IFERROR(C14/B14,0)</f>
         <v/>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="6">
         <f>ROUND(B14/26,0)</f>
         <v/>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="6">
         <f>IF(E14&gt;=1,"🟢 On Target",IF(E14&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>HARINDER</t>
-        </is>
-      </c>
-      <c r="B15" s="5">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Saha Travnook</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
         <f>'Weekly Tracker'!C11</f>
         <v/>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="6">
         <f>'Weekly Tracker'!AS11</f>
         <v/>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="6">
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="6">
         <f>IFERROR(C15/B15,0)</f>
         <v/>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="6">
         <f>ROUND(B15/26,0)</f>
         <v/>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="6">
         <f>IF(E15&gt;=1,"🟢 On Target",IF(E15&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
@@ -853,54 +852,118 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>TEAM TOTAL</t>
-        </is>
-      </c>
-      <c r="B16" s="7">
-        <f>SUM(B10:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="7">
-        <f>SUM(C10:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="7">
+          <t>Alshimaa Ahmed</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>'Weekly Tracker'!C12</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>'Weekly Tracker'!AS12</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="6">
         <f>IFERROR(C16/B16,0)</f>
         <v/>
       </c>
-      <c r="F16" s="7">
-        <f>SUM(F10:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="7">
+      <c r="F16" s="6">
+        <f>ROUND(B16/26,0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="6">
         <f>IF(E16&gt;=1,"🟢 On Target",IF(E16&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Khozema Nogamawala</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <f>'Weekly Tracker'!C13</f>
+        <v/>
+      </c>
+      <c r="C17" s="6">
+        <f>'Weekly Tracker'!AS13</f>
+        <v/>
+      </c>
+      <c r="D17" s="6">
+        <f>B17-C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="6">
+        <f>IFERROR(C17/B17,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="6">
+        <f>ROUND(B17/26,0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="6">
+        <f>IF(E17&gt;=1,"🟢 On Target",IF(E17&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>ℹ️  Each agent's monthly target is a flat AED 25,000 (6 agents × 25,000 = AED 150,000 team target). Yellow cells on 'Weekly Tracker' = daily entry; everything else here updates automatically.</t>
+          <t>TEAM TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>SUM(B10:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="8">
+        <f>SUM(C10:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="8">
+        <f>B18-C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="8">
+        <f>IFERROR(C18/B18,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="8">
+        <f>SUM(F10:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="8">
+        <f>IF(E18&gt;=1,"🟢 On Target",IF(E18&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>ℹ️  Each agent's base target is a flat AED 25,000 (8 agents × 25,000 = AED 200,000 combined individual targets). The team target (cell A6, AED 170,000) is set independently as the overall business goal, so it need not equal the combined individual targets. Yellow cells on 'Weekly Tracker' = daily entry; everything else here updates automatically.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A18:H18"/>
+  <mergeCells count="14">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="G16:H16"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="G11:H11"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G18:H18"/>
     <mergeCell ref="A8:H8"/>
+    <mergeCell ref="G17:H17"/>
     <mergeCell ref="G13:H13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -913,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV14"/>
+  <dimension ref="A1:AV16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -967,7 +1030,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>TRAVNOOK TRAVELS — SEPTEMBER 2026  WEEKLY &amp; MONTHLY TRACKER</t>
         </is>
@@ -976,14 +1039,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Team Lead: Bindhya   |   Monthly Target: AED 25,000 per agent   |   Working Days: 26   |   🟡 Yellow cells = daily data entry</t>
+          <t>Team Lead: Bindhya Travnook   |   Team Target: AED 170,000   |   Per-Agent Base Target: AED 25,000   |   Working Days: 26   |   🟡 Yellow cells = daily data entry</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>⚠️  Mid-month checkpoint: be at AED 10,577 per agent (AED 63,462 team) by 12 Sep / end of WK 2 to avoid a month-end rush.</t>
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>⚠️  Mid-month checkpoint: each agent aim AED 10,577 (base-target pacing)   |   Team aim AED 71,923 against the AED 170,000 team target   by 12 Sep / end of WK 2.</t>
         </is>
       </c>
     </row>
@@ -1086,247 +1149,247 @@
       </c>
     </row>
     <row r="5" ht="27.75" customHeight="1">
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>WK
 TARGET</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Sep 1
 Tue</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Sep 2
 Wed</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Sep 3
 Thu</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>Sep 4
 Fri</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>Sep 5
 Sat</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>WK
 ACHIEVED</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>WK
 DEFICIT</t>
         </is>
       </c>
-      <c r="L5" s="11" t="inlineStr">
+      <c r="L5" s="12" t="inlineStr">
         <is>
           <t>WK
 TARGET</t>
         </is>
       </c>
-      <c r="M5" s="11" t="inlineStr">
+      <c r="M5" s="12" t="inlineStr">
         <is>
           <t>Sep 7
 Mon</t>
         </is>
       </c>
-      <c r="N5" s="11" t="inlineStr">
+      <c r="N5" s="12" t="inlineStr">
         <is>
           <t>Sep 8
 Tue</t>
         </is>
       </c>
-      <c r="O5" s="11" t="inlineStr">
+      <c r="O5" s="12" t="inlineStr">
         <is>
           <t>Sep 9
 Wed</t>
         </is>
       </c>
-      <c r="P5" s="11" t="inlineStr">
+      <c r="P5" s="12" t="inlineStr">
         <is>
           <t>Sep 10
 Thu</t>
         </is>
       </c>
-      <c r="Q5" s="11" t="inlineStr">
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>Sep 11
 Fri</t>
         </is>
       </c>
-      <c r="R5" s="11" t="inlineStr">
+      <c r="R5" s="12" t="inlineStr">
         <is>
           <t>Sep 12
 Sat</t>
         </is>
       </c>
-      <c r="S5" s="11" t="inlineStr">
+      <c r="S5" s="12" t="inlineStr">
         <is>
           <t>WK
 ACHIEVED</t>
         </is>
       </c>
-      <c r="T5" s="11" t="inlineStr">
+      <c r="T5" s="12" t="inlineStr">
         <is>
           <t>WK
 DEFICIT</t>
         </is>
       </c>
-      <c r="U5" s="11" t="inlineStr">
+      <c r="U5" s="12" t="inlineStr">
         <is>
           <t>WK
 TARGET</t>
         </is>
       </c>
-      <c r="V5" s="11" t="inlineStr">
+      <c r="V5" s="12" t="inlineStr">
         <is>
           <t>Sep 14
 Mon</t>
         </is>
       </c>
-      <c r="W5" s="11" t="inlineStr">
+      <c r="W5" s="12" t="inlineStr">
         <is>
           <t>Sep 15
 Tue</t>
         </is>
       </c>
-      <c r="X5" s="11" t="inlineStr">
+      <c r="X5" s="12" t="inlineStr">
         <is>
           <t>Sep 16
 Wed</t>
         </is>
       </c>
-      <c r="Y5" s="11" t="inlineStr">
+      <c r="Y5" s="12" t="inlineStr">
         <is>
           <t>Sep 17
 Thu</t>
         </is>
       </c>
-      <c r="Z5" s="11" t="inlineStr">
+      <c r="Z5" s="12" t="inlineStr">
         <is>
           <t>Sep 18
 Fri</t>
         </is>
       </c>
-      <c r="AA5" s="11" t="inlineStr">
+      <c r="AA5" s="12" t="inlineStr">
         <is>
           <t>Sep 19
 Sat</t>
         </is>
       </c>
-      <c r="AB5" s="11" t="inlineStr">
+      <c r="AB5" s="12" t="inlineStr">
         <is>
           <t>WK
 ACHIEVED</t>
         </is>
       </c>
-      <c r="AC5" s="11" t="inlineStr">
+      <c r="AC5" s="12" t="inlineStr">
         <is>
           <t>WK
 DEFICIT</t>
         </is>
       </c>
-      <c r="AD5" s="11" t="inlineStr">
+      <c r="AD5" s="12" t="inlineStr">
         <is>
           <t>WK
 TARGET</t>
         </is>
       </c>
-      <c r="AE5" s="11" t="inlineStr">
+      <c r="AE5" s="12" t="inlineStr">
         <is>
           <t>Sep 21
 Mon</t>
         </is>
       </c>
-      <c r="AF5" s="11" t="inlineStr">
+      <c r="AF5" s="12" t="inlineStr">
         <is>
           <t>Sep 22
 Tue</t>
         </is>
       </c>
-      <c r="AG5" s="11" t="inlineStr">
+      <c r="AG5" s="12" t="inlineStr">
         <is>
           <t>Sep 23
 Wed</t>
         </is>
       </c>
-      <c r="AH5" s="11" t="inlineStr">
+      <c r="AH5" s="12" t="inlineStr">
         <is>
           <t>Sep 24
 Thu</t>
         </is>
       </c>
-      <c r="AI5" s="11" t="inlineStr">
+      <c r="AI5" s="12" t="inlineStr">
         <is>
           <t>Sep 25
 Fri</t>
         </is>
       </c>
-      <c r="AJ5" s="11" t="inlineStr">
+      <c r="AJ5" s="12" t="inlineStr">
         <is>
           <t>Sep 26
 Sat</t>
         </is>
       </c>
-      <c r="AK5" s="11" t="inlineStr">
+      <c r="AK5" s="12" t="inlineStr">
         <is>
           <t>WK
 ACHIEVED</t>
         </is>
       </c>
-      <c r="AL5" s="11" t="inlineStr">
+      <c r="AL5" s="12" t="inlineStr">
         <is>
           <t>WK
 DEFICIT</t>
         </is>
       </c>
-      <c r="AM5" s="11" t="inlineStr">
+      <c r="AM5" s="12" t="inlineStr">
         <is>
           <t>WK
 TARGET</t>
         </is>
       </c>
-      <c r="AN5" s="11" t="inlineStr">
+      <c r="AN5" s="12" t="inlineStr">
         <is>
           <t>Sep 28
 Mon</t>
         </is>
       </c>
-      <c r="AO5" s="11" t="inlineStr">
+      <c r="AO5" s="12" t="inlineStr">
         <is>
           <t>Sep 29
 Tue</t>
         </is>
       </c>
-      <c r="AP5" s="11" t="inlineStr">
+      <c r="AP5" s="12" t="inlineStr">
         <is>
           <t>Sep 30
 Wed</t>
         </is>
       </c>
-      <c r="AQ5" s="11" t="inlineStr">
+      <c r="AQ5" s="12" t="inlineStr">
         <is>
           <t>WK
 ACHIEVED</t>
         </is>
       </c>
-      <c r="AR5" s="11" t="inlineStr">
+      <c r="AR5" s="12" t="inlineStr">
         <is>
           <t>WK
 DEFICIT</t>
@@ -1334,19 +1397,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>SAHA</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Iyan</t>
+        </is>
+      </c>
+      <c r="B6" s="6">
         <f>ROUND(C6/26,0)</f>
         <v/>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="6">
         <f>ROUND($C6*5/26,0)</f>
         <v/>
       </c>
@@ -1365,15 +1428,15 @@
       <c r="I6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="6">
         <f>SUM(E6:I6)</f>
         <v/>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="6">
         <f>D6-J6</f>
         <v/>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="6">
         <f>ROUND($C6*6/26,0)</f>
         <v/>
       </c>
@@ -1395,15 +1458,15 @@
       <c r="R6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="S6" s="5">
+      <c r="S6" s="6">
         <f>SUM(M6:R6)</f>
         <v/>
       </c>
-      <c r="T6" s="5">
+      <c r="T6" s="6">
         <f>L6-S6</f>
         <v/>
       </c>
-      <c r="U6" s="5">
+      <c r="U6" s="6">
         <f>ROUND($C6*6/26,0)</f>
         <v/>
       </c>
@@ -1425,15 +1488,15 @@
       <c r="AA6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AB6" s="5">
+      <c r="AB6" s="6">
         <f>SUM(V6:AA6)</f>
         <v/>
       </c>
-      <c r="AC6" s="5">
+      <c r="AC6" s="6">
         <f>U6-AB6</f>
         <v/>
       </c>
-      <c r="AD6" s="5">
+      <c r="AD6" s="6">
         <f>ROUND($C6*6/26,0)</f>
         <v/>
       </c>
@@ -1455,15 +1518,15 @@
       <c r="AJ6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AK6" s="5">
+      <c r="AK6" s="6">
         <f>SUM(AE6:AJ6)</f>
         <v/>
       </c>
-      <c r="AL6" s="5">
+      <c r="AL6" s="6">
         <f>AD6-AK6</f>
         <v/>
       </c>
-      <c r="AM6" s="5">
+      <c r="AM6" s="6">
         <f>ROUND($C6*3/26,0)</f>
         <v/>
       </c>
@@ -1476,45 +1539,45 @@
       <c r="AP6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AQ6" s="5">
+      <c r="AQ6" s="6">
         <f>SUM(AN6:AP6)</f>
         <v/>
       </c>
-      <c r="AR6" s="5">
+      <c r="AR6" s="6">
         <f>AM6-AQ6</f>
         <v/>
       </c>
-      <c r="AS6" s="5">
+      <c r="AS6" s="6">
         <f>J6+S6+AB6+AK6+AQ6</f>
         <v/>
       </c>
-      <c r="AT6" s="5">
+      <c r="AT6" s="6">
         <f>C6-AS6</f>
         <v/>
       </c>
-      <c r="AU6" s="5">
+      <c r="AU6" s="6">
         <f>IFERROR(AS6/C6,0)</f>
         <v/>
       </c>
-      <c r="AV6" s="5">
+      <c r="AV6" s="6">
         <f>IF(AU6&gt;=1,"🟢 On Target",IF(AU6&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>IYAD</t>
-        </is>
-      </c>
-      <c r="B7" s="5">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Harinder</t>
+        </is>
+      </c>
+      <c r="B7" s="6">
         <f>ROUND(C7/26,0)</f>
         <v/>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="6">
         <f>ROUND($C7*5/26,0)</f>
         <v/>
       </c>
@@ -1533,15 +1596,15 @@
       <c r="I7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="6">
         <f>SUM(E7:I7)</f>
         <v/>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="6">
         <f>D7-J7</f>
         <v/>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="6">
         <f>ROUND($C7*6/26,0)</f>
         <v/>
       </c>
@@ -1563,15 +1626,15 @@
       <c r="R7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="S7" s="5">
+      <c r="S7" s="6">
         <f>SUM(M7:R7)</f>
         <v/>
       </c>
-      <c r="T7" s="5">
+      <c r="T7" s="6">
         <f>L7-S7</f>
         <v/>
       </c>
-      <c r="U7" s="5">
+      <c r="U7" s="6">
         <f>ROUND($C7*6/26,0)</f>
         <v/>
       </c>
@@ -1593,15 +1656,15 @@
       <c r="AA7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AB7" s="5">
+      <c r="AB7" s="6">
         <f>SUM(V7:AA7)</f>
         <v/>
       </c>
-      <c r="AC7" s="5">
+      <c r="AC7" s="6">
         <f>U7-AB7</f>
         <v/>
       </c>
-      <c r="AD7" s="5">
+      <c r="AD7" s="6">
         <f>ROUND($C7*6/26,0)</f>
         <v/>
       </c>
@@ -1623,15 +1686,15 @@
       <c r="AJ7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AK7" s="5">
+      <c r="AK7" s="6">
         <f>SUM(AE7:AJ7)</f>
         <v/>
       </c>
-      <c r="AL7" s="5">
+      <c r="AL7" s="6">
         <f>AD7-AK7</f>
         <v/>
       </c>
-      <c r="AM7" s="5">
+      <c r="AM7" s="6">
         <f>ROUND($C7*3/26,0)</f>
         <v/>
       </c>
@@ -1644,45 +1707,45 @@
       <c r="AP7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AQ7" s="5">
+      <c r="AQ7" s="6">
         <f>SUM(AN7:AP7)</f>
         <v/>
       </c>
-      <c r="AR7" s="5">
+      <c r="AR7" s="6">
         <f>AM7-AQ7</f>
         <v/>
       </c>
-      <c r="AS7" s="5">
+      <c r="AS7" s="6">
         <f>J7+S7+AB7+AK7+AQ7</f>
         <v/>
       </c>
-      <c r="AT7" s="5">
+      <c r="AT7" s="6">
         <f>C7-AS7</f>
         <v/>
       </c>
-      <c r="AU7" s="5">
+      <c r="AU7" s="6">
         <f>IFERROR(AS7/C7,0)</f>
         <v/>
       </c>
-      <c r="AV7" s="5">
+      <c r="AV7" s="6">
         <f>IF(AU7&gt;=1,"🟢 On Target",IF(AU7&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>RIHAB</t>
-        </is>
-      </c>
-      <c r="B8" s="5">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Rihab Travnook</t>
+        </is>
+      </c>
+      <c r="B8" s="6">
         <f>ROUND(C8/26,0)</f>
         <v/>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="6">
         <f>ROUND($C8*5/26,0)</f>
         <v/>
       </c>
@@ -1701,15 +1764,15 @@
       <c r="I8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="6">
         <f>SUM(E8:I8)</f>
         <v/>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="6">
         <f>D8-J8</f>
         <v/>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="6">
         <f>ROUND($C8*6/26,0)</f>
         <v/>
       </c>
@@ -1731,15 +1794,15 @@
       <c r="R8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="S8" s="5">
+      <c r="S8" s="6">
         <f>SUM(M8:R8)</f>
         <v/>
       </c>
-      <c r="T8" s="5">
+      <c r="T8" s="6">
         <f>L8-S8</f>
         <v/>
       </c>
-      <c r="U8" s="5">
+      <c r="U8" s="6">
         <f>ROUND($C8*6/26,0)</f>
         <v/>
       </c>
@@ -1761,15 +1824,15 @@
       <c r="AA8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AB8" s="5">
+      <c r="AB8" s="6">
         <f>SUM(V8:AA8)</f>
         <v/>
       </c>
-      <c r="AC8" s="5">
+      <c r="AC8" s="6">
         <f>U8-AB8</f>
         <v/>
       </c>
-      <c r="AD8" s="5">
+      <c r="AD8" s="6">
         <f>ROUND($C8*6/26,0)</f>
         <v/>
       </c>
@@ -1791,15 +1854,15 @@
       <c r="AJ8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AK8" s="5">
+      <c r="AK8" s="6">
         <f>SUM(AE8:AJ8)</f>
         <v/>
       </c>
-      <c r="AL8" s="5">
+      <c r="AL8" s="6">
         <f>AD8-AK8</f>
         <v/>
       </c>
-      <c r="AM8" s="5">
+      <c r="AM8" s="6">
         <f>ROUND($C8*3/26,0)</f>
         <v/>
       </c>
@@ -1812,45 +1875,45 @@
       <c r="AP8" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AQ8" s="5">
+      <c r="AQ8" s="6">
         <f>SUM(AN8:AP8)</f>
         <v/>
       </c>
-      <c r="AR8" s="5">
+      <c r="AR8" s="6">
         <f>AM8-AQ8</f>
         <v/>
       </c>
-      <c r="AS8" s="5">
+      <c r="AS8" s="6">
         <f>J8+S8+AB8+AK8+AQ8</f>
         <v/>
       </c>
-      <c r="AT8" s="5">
+      <c r="AT8" s="6">
         <f>C8-AS8</f>
         <v/>
       </c>
-      <c r="AU8" s="5">
+      <c r="AU8" s="6">
         <f>IFERROR(AS8/C8,0)</f>
         <v/>
       </c>
-      <c r="AV8" s="5">
+      <c r="AV8" s="6">
         <f>IF(AU8&gt;=1,"🟢 On Target",IF(AU8&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>SHILPA</t>
-        </is>
-      </c>
-      <c r="B9" s="5">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Ibrahim Travnook</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
         <f>ROUND(C9/26,0)</f>
         <v/>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="6">
         <f>ROUND($C9*5/26,0)</f>
         <v/>
       </c>
@@ -1869,15 +1932,15 @@
       <c r="I9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="6">
         <f>SUM(E9:I9)</f>
         <v/>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="6">
         <f>D9-J9</f>
         <v/>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="6">
         <f>ROUND($C9*6/26,0)</f>
         <v/>
       </c>
@@ -1899,15 +1962,15 @@
       <c r="R9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="S9" s="5">
+      <c r="S9" s="6">
         <f>SUM(M9:R9)</f>
         <v/>
       </c>
-      <c r="T9" s="5">
+      <c r="T9" s="6">
         <f>L9-S9</f>
         <v/>
       </c>
-      <c r="U9" s="5">
+      <c r="U9" s="6">
         <f>ROUND($C9*6/26,0)</f>
         <v/>
       </c>
@@ -1929,15 +1992,15 @@
       <c r="AA9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" s="5">
+      <c r="AB9" s="6">
         <f>SUM(V9:AA9)</f>
         <v/>
       </c>
-      <c r="AC9" s="5">
+      <c r="AC9" s="6">
         <f>U9-AB9</f>
         <v/>
       </c>
-      <c r="AD9" s="5">
+      <c r="AD9" s="6">
         <f>ROUND($C9*6/26,0)</f>
         <v/>
       </c>
@@ -1959,15 +2022,15 @@
       <c r="AJ9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AK9" s="5">
+      <c r="AK9" s="6">
         <f>SUM(AE9:AJ9)</f>
         <v/>
       </c>
-      <c r="AL9" s="5">
+      <c r="AL9" s="6">
         <f>AD9-AK9</f>
         <v/>
       </c>
-      <c r="AM9" s="5">
+      <c r="AM9" s="6">
         <f>ROUND($C9*3/26,0)</f>
         <v/>
       </c>
@@ -1980,45 +2043,45 @@
       <c r="AP9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AQ9" s="5">
+      <c r="AQ9" s="6">
         <f>SUM(AN9:AP9)</f>
         <v/>
       </c>
-      <c r="AR9" s="5">
+      <c r="AR9" s="6">
         <f>AM9-AQ9</f>
         <v/>
       </c>
-      <c r="AS9" s="5">
+      <c r="AS9" s="6">
         <f>J9+S9+AB9+AK9+AQ9</f>
         <v/>
       </c>
-      <c r="AT9" s="5">
+      <c r="AT9" s="6">
         <f>C9-AS9</f>
         <v/>
       </c>
-      <c r="AU9" s="5">
+      <c r="AU9" s="6">
         <f>IFERROR(AS9/C9,0)</f>
         <v/>
       </c>
-      <c r="AV9" s="5">
+      <c r="AV9" s="6">
         <f>IF(AU9&gt;=1,"🟢 On Target",IF(AU9&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>ALSHIMAA</t>
-        </is>
-      </c>
-      <c r="B10" s="5">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Chaimaa Benchohra</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
         <f>ROUND(C10/26,0)</f>
         <v/>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="6">
         <f>ROUND($C10*5/26,0)</f>
         <v/>
       </c>
@@ -2037,15 +2100,15 @@
       <c r="I10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="6">
         <f>SUM(E10:I10)</f>
         <v/>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="6">
         <f>D10-J10</f>
         <v/>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="6">
         <f>ROUND($C10*6/26,0)</f>
         <v/>
       </c>
@@ -2067,15 +2130,15 @@
       <c r="R10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="S10" s="5">
+      <c r="S10" s="6">
         <f>SUM(M10:R10)</f>
         <v/>
       </c>
-      <c r="T10" s="5">
+      <c r="T10" s="6">
         <f>L10-S10</f>
         <v/>
       </c>
-      <c r="U10" s="5">
+      <c r="U10" s="6">
         <f>ROUND($C10*6/26,0)</f>
         <v/>
       </c>
@@ -2097,15 +2160,15 @@
       <c r="AA10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AB10" s="5">
+      <c r="AB10" s="6">
         <f>SUM(V10:AA10)</f>
         <v/>
       </c>
-      <c r="AC10" s="5">
+      <c r="AC10" s="6">
         <f>U10-AB10</f>
         <v/>
       </c>
-      <c r="AD10" s="5">
+      <c r="AD10" s="6">
         <f>ROUND($C10*6/26,0)</f>
         <v/>
       </c>
@@ -2127,15 +2190,15 @@
       <c r="AJ10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AK10" s="5">
+      <c r="AK10" s="6">
         <f>SUM(AE10:AJ10)</f>
         <v/>
       </c>
-      <c r="AL10" s="5">
+      <c r="AL10" s="6">
         <f>AD10-AK10</f>
         <v/>
       </c>
-      <c r="AM10" s="5">
+      <c r="AM10" s="6">
         <f>ROUND($C10*3/26,0)</f>
         <v/>
       </c>
@@ -2148,45 +2211,45 @@
       <c r="AP10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AQ10" s="5">
+      <c r="AQ10" s="6">
         <f>SUM(AN10:AP10)</f>
         <v/>
       </c>
-      <c r="AR10" s="5">
+      <c r="AR10" s="6">
         <f>AM10-AQ10</f>
         <v/>
       </c>
-      <c r="AS10" s="5">
+      <c r="AS10" s="6">
         <f>J10+S10+AB10+AK10+AQ10</f>
         <v/>
       </c>
-      <c r="AT10" s="5">
+      <c r="AT10" s="6">
         <f>C10-AS10</f>
         <v/>
       </c>
-      <c r="AU10" s="5">
+      <c r="AU10" s="6">
         <f>IFERROR(AS10/C10,0)</f>
         <v/>
       </c>
-      <c r="AV10" s="5">
+      <c r="AV10" s="6">
         <f>IF(AU10&gt;=1,"🟢 On Target",IF(AU10&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>HARINDER</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Saha Travnook</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
         <f>ROUND(C11/26,0)</f>
         <v/>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="6">
         <f>ROUND($C11*5/26,0)</f>
         <v/>
       </c>
@@ -2205,15 +2268,15 @@
       <c r="I11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="6">
         <f>SUM(E11:I11)</f>
         <v/>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="6">
         <f>D11-J11</f>
         <v/>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="6">
         <f>ROUND($C11*6/26,0)</f>
         <v/>
       </c>
@@ -2235,15 +2298,15 @@
       <c r="R11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="S11" s="5">
+      <c r="S11" s="6">
         <f>SUM(M11:R11)</f>
         <v/>
       </c>
-      <c r="T11" s="5">
+      <c r="T11" s="6">
         <f>L11-S11</f>
         <v/>
       </c>
-      <c r="U11" s="5">
+      <c r="U11" s="6">
         <f>ROUND($C11*6/26,0)</f>
         <v/>
       </c>
@@ -2265,15 +2328,15 @@
       <c r="AA11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AB11" s="5">
+      <c r="AB11" s="6">
         <f>SUM(V11:AA11)</f>
         <v/>
       </c>
-      <c r="AC11" s="5">
+      <c r="AC11" s="6">
         <f>U11-AB11</f>
         <v/>
       </c>
-      <c r="AD11" s="5">
+      <c r="AD11" s="6">
         <f>ROUND($C11*6/26,0)</f>
         <v/>
       </c>
@@ -2295,15 +2358,15 @@
       <c r="AJ11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AK11" s="5">
+      <c r="AK11" s="6">
         <f>SUM(AE11:AJ11)</f>
         <v/>
       </c>
-      <c r="AL11" s="5">
+      <c r="AL11" s="6">
         <f>AD11-AK11</f>
         <v/>
       </c>
-      <c r="AM11" s="5">
+      <c r="AM11" s="6">
         <f>ROUND($C11*3/26,0)</f>
         <v/>
       </c>
@@ -2316,130 +2379,466 @@
       <c r="AP11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="AQ11" s="5">
+      <c r="AQ11" s="6">
         <f>SUM(AN11:AP11)</f>
         <v/>
       </c>
-      <c r="AR11" s="5">
+      <c r="AR11" s="6">
         <f>AM11-AQ11</f>
         <v/>
       </c>
-      <c r="AS11" s="5">
+      <c r="AS11" s="6">
         <f>J11+S11+AB11+AK11+AQ11</f>
         <v/>
       </c>
-      <c r="AT11" s="5">
+      <c r="AT11" s="6">
         <f>C11-AS11</f>
         <v/>
       </c>
-      <c r="AU11" s="5">
+      <c r="AU11" s="6">
         <f>IFERROR(AS11/C11,0)</f>
         <v/>
       </c>
-      <c r="AV11" s="5">
+      <c r="AV11" s="6">
         <f>IF(AU11&gt;=1,"🟢 On Target",IF(AU11&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Alshimaa Ahmed</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <f>ROUND(C12/26,0)</f>
+        <v/>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D12" s="6">
+        <f>ROUND($C12*5/26,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <f>SUM(E12:I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="6">
+        <f>D12-J12</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>ROUND($C12*6/26,0)</f>
+        <v/>
+      </c>
+      <c r="M12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="6">
+        <f>SUM(M12:R12)</f>
+        <v/>
+      </c>
+      <c r="T12" s="6">
+        <f>L12-S12</f>
+        <v/>
+      </c>
+      <c r="U12" s="6">
+        <f>ROUND($C12*6/26,0)</f>
+        <v/>
+      </c>
+      <c r="V12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="6">
+        <f>SUM(V12:AA12)</f>
+        <v/>
+      </c>
+      <c r="AC12" s="6">
+        <f>U12-AB12</f>
+        <v/>
+      </c>
+      <c r="AD12" s="6">
+        <f>ROUND($C12*6/26,0)</f>
+        <v/>
+      </c>
+      <c r="AE12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" s="6">
+        <f>SUM(AE12:AJ12)</f>
+        <v/>
+      </c>
+      <c r="AL12" s="6">
+        <f>AD12-AK12</f>
+        <v/>
+      </c>
+      <c r="AM12" s="6">
+        <f>ROUND($C12*3/26,0)</f>
+        <v/>
+      </c>
+      <c r="AN12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ12" s="6">
+        <f>SUM(AN12:AP12)</f>
+        <v/>
+      </c>
+      <c r="AR12" s="6">
+        <f>AM12-AQ12</f>
+        <v/>
+      </c>
+      <c r="AS12" s="6">
+        <f>J12+S12+AB12+AK12+AQ12</f>
+        <v/>
+      </c>
+      <c r="AT12" s="6">
+        <f>C12-AS12</f>
+        <v/>
+      </c>
+      <c r="AU12" s="6">
+        <f>IFERROR(AS12/C12,0)</f>
+        <v/>
+      </c>
+      <c r="AV12" s="6">
+        <f>IF(AU12&gt;=1,"🟢 On Target",IF(AU12&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Khozema Nogamawala</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <f>ROUND(C13/26,0)</f>
+        <v/>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D13" s="6">
+        <f>ROUND($C13*5/26,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6">
+        <f>SUM(E13:I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="6">
+        <f>D13-J13</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>ROUND($C13*6/26,0)</f>
+        <v/>
+      </c>
+      <c r="M13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="6">
+        <f>SUM(M13:R13)</f>
+        <v/>
+      </c>
+      <c r="T13" s="6">
+        <f>L13-S13</f>
+        <v/>
+      </c>
+      <c r="U13" s="6">
+        <f>ROUND($C13*6/26,0)</f>
+        <v/>
+      </c>
+      <c r="V13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="6">
+        <f>SUM(V13:AA13)</f>
+        <v/>
+      </c>
+      <c r="AC13" s="6">
+        <f>U13-AB13</f>
+        <v/>
+      </c>
+      <c r="AD13" s="6">
+        <f>ROUND($C13*6/26,0)</f>
+        <v/>
+      </c>
+      <c r="AE13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" s="6">
+        <f>SUM(AE13:AJ13)</f>
+        <v/>
+      </c>
+      <c r="AL13" s="6">
+        <f>AD13-AK13</f>
+        <v/>
+      </c>
+      <c r="AM13" s="6">
+        <f>ROUND($C13*3/26,0)</f>
+        <v/>
+      </c>
+      <c r="AN13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ13" s="6">
+        <f>SUM(AN13:AP13)</f>
+        <v/>
+      </c>
+      <c r="AR13" s="6">
+        <f>AM13-AQ13</f>
+        <v/>
+      </c>
+      <c r="AS13" s="6">
+        <f>J13+S13+AB13+AK13+AQ13</f>
+        <v/>
+      </c>
+      <c r="AT13" s="6">
+        <f>C13-AS13</f>
+        <v/>
+      </c>
+      <c r="AU13" s="6">
+        <f>IFERROR(AS13/C13,0)</f>
+        <v/>
+      </c>
+      <c r="AV13" s="6">
+        <f>IF(AU13&gt;=1,"🟢 On Target",IF(AU13&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>TEAM TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="7">
-        <f>SUM(B6:B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="7">
-        <f>SUM(C6:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="7">
-        <f>SUM(D6:D11)</f>
-        <v/>
-      </c>
-      <c r="J12" s="7">
-        <f>SUM(J6:J11)</f>
-        <v/>
-      </c>
-      <c r="K12" s="7">
-        <f>SUM(K6:K11)</f>
-        <v/>
-      </c>
-      <c r="L12" s="7">
-        <f>SUM(L6:L11)</f>
-        <v/>
-      </c>
-      <c r="S12" s="7">
-        <f>SUM(S6:S11)</f>
-        <v/>
-      </c>
-      <c r="T12" s="7">
-        <f>SUM(T6:T11)</f>
-        <v/>
-      </c>
-      <c r="U12" s="7">
-        <f>SUM(U6:U11)</f>
-        <v/>
-      </c>
-      <c r="AB12" s="7">
-        <f>SUM(AB6:AB11)</f>
-        <v/>
-      </c>
-      <c r="AC12" s="7">
-        <f>SUM(AC6:AC11)</f>
-        <v/>
-      </c>
-      <c r="AD12" s="7">
-        <f>SUM(AD6:AD11)</f>
-        <v/>
-      </c>
-      <c r="AK12" s="7">
-        <f>SUM(AK6:AK11)</f>
-        <v/>
-      </c>
-      <c r="AL12" s="7">
-        <f>SUM(AL6:AL11)</f>
-        <v/>
-      </c>
-      <c r="AM12" s="7">
-        <f>SUM(AM6:AM11)</f>
-        <v/>
-      </c>
-      <c r="AQ12" s="7">
-        <f>SUM(AQ6:AQ11)</f>
-        <v/>
-      </c>
-      <c r="AR12" s="7">
-        <f>SUM(AR6:AR11)</f>
-        <v/>
-      </c>
-      <c r="AS12" s="7">
-        <f>SUM(AS6:AS11)</f>
-        <v/>
-      </c>
-      <c r="AT12" s="7">
-        <f>SUM(AT6:AT11)</f>
-        <v/>
-      </c>
-      <c r="AU12" s="7">
-        <f>IFERROR(AS12/C12,0)</f>
-        <v/>
-      </c>
-      <c r="AV12" s="7">
-        <f>IF(AU12&gt;=1,"🟢 On Target",IF(AU12&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="B14" s="8">
+        <f>SUM(B6:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="8">
+        <f>SUM(C6:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>SUM(D6:D13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="8">
+        <f>SUM(J6:J13)</f>
+        <v/>
+      </c>
+      <c r="K14" s="8">
+        <f>SUM(K6:K13)</f>
+        <v/>
+      </c>
+      <c r="L14" s="8">
+        <f>SUM(L6:L13)</f>
+        <v/>
+      </c>
+      <c r="S14" s="8">
+        <f>SUM(S6:S13)</f>
+        <v/>
+      </c>
+      <c r="T14" s="8">
+        <f>SUM(T6:T13)</f>
+        <v/>
+      </c>
+      <c r="U14" s="8">
+        <f>SUM(U6:U13)</f>
+        <v/>
+      </c>
+      <c r="AB14" s="8">
+        <f>SUM(AB6:AB13)</f>
+        <v/>
+      </c>
+      <c r="AC14" s="8">
+        <f>SUM(AC6:AC13)</f>
+        <v/>
+      </c>
+      <c r="AD14" s="8">
+        <f>SUM(AD6:AD13)</f>
+        <v/>
+      </c>
+      <c r="AK14" s="8">
+        <f>SUM(AK6:AK13)</f>
+        <v/>
+      </c>
+      <c r="AL14" s="8">
+        <f>SUM(AL6:AL13)</f>
+        <v/>
+      </c>
+      <c r="AM14" s="8">
+        <f>SUM(AM6:AM13)</f>
+        <v/>
+      </c>
+      <c r="AQ14" s="8">
+        <f>SUM(AQ6:AQ13)</f>
+        <v/>
+      </c>
+      <c r="AR14" s="8">
+        <f>SUM(AR6:AR13)</f>
+        <v/>
+      </c>
+      <c r="AS14" s="8">
+        <f>SUM(AS6:AS13)</f>
+        <v/>
+      </c>
+      <c r="AT14" s="8">
+        <f>SUM(AT6:AT13)</f>
+        <v/>
+      </c>
+      <c r="AU14" s="8">
+        <f>IFERROR(AS14/C14,0)</f>
+        <v/>
+      </c>
+      <c r="AV14" s="8">
+        <f>IF(AU14&gt;=1,"🟢 On Target",IF(AU14&gt;=0.7,"🟡 Watch","🔴 Critical"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>MID-MONTH CHECKPOINT (through 12 Sep / WK1–WK2)</t>
         </is>
       </c>
-      <c r="D14" s="10">
-        <f>"Team actual: AED "&amp;TEXT(J12+S12,"#,##0")&amp;"   |   Aim: AED 63,462 team (AED 10,577/agent)"</f>
+      <c r="D16" s="11">
+        <f>"Team actual: AED "&amp;TEXT(J14+S14,"#,##0")&amp;"   |   Aim: AED 71,923 team (against AED 170,000 team target)"</f>
         <v/>
       </c>
     </row>
@@ -2447,11 +2846,10 @@
   <mergeCells count="17">
     <mergeCell ref="L4:T4"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="D14:AV14"/>
     <mergeCell ref="A1:AV1"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A16:C16"/>
     <mergeCell ref="AV4:AV5"/>
     <mergeCell ref="AT4:AT5"/>
     <mergeCell ref="AU4:AU5"/>
@@ -2459,6 +2857,7 @@
     <mergeCell ref="AD4:AL4"/>
     <mergeCell ref="AM4:AR4"/>
     <mergeCell ref="AS4:AS5"/>
+    <mergeCell ref="D16:AV16"/>
     <mergeCell ref="U4:AC4"/>
     <mergeCell ref="D4:K4"/>
     <mergeCell ref="A2:AV2"/>

</xml_diff>